<commit_message>
dev/added annualized roi for exchange assets
</commit_message>
<xml_diff>
--- a/xtb/HistoriaTransakcji.xlsx
+++ b/xtb/HistoriaTransakcji.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d98d39ada2f13ae1/Desktop/Foldery/Finanse osobiste/portfolio-management/xtb/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natal\Desktop\Codes\python\portfolio-management\xtb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_2B5928CF928B565EB1717DD2576050B07B63F60C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A274607E-AE76-4A74-89E1-54ADD413AAFB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44D3CB7A-FBEF-4371-B843-CB52AA447FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Transactions" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="30">
   <si>
     <t>ticker</t>
   </si>
@@ -98,6 +98,18 @@
   </si>
   <si>
     <t>timestamp</t>
+  </si>
+  <si>
+    <t>2026-05-11T16:07:00</t>
+  </si>
+  <si>
+    <t>2026-06-12T14:18:00</t>
+  </si>
+  <si>
+    <t>2026-05-11T16:31:00</t>
+  </si>
+  <si>
+    <t>2026-06-12T13:41:00</t>
   </si>
 </sst>
 </file>
@@ -452,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="9" width="20" customWidth="1"/>
@@ -593,25 +605,25 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
         <v>9</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="D6">
-        <v>1.9616</v>
+        <v>3.6387</v>
       </c>
       <c r="E6">
-        <v>229.37</v>
+        <v>128.80000000000001</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>4.2601000000000004</v>
       </c>
       <c r="G6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
@@ -619,25 +631,25 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="D7">
-        <v>11.824199999999999</v>
+        <v>6.0006000000000004</v>
       </c>
       <c r="E7">
-        <v>230.6</v>
+        <v>117.09</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>4.2694000000000001</v>
       </c>
       <c r="G7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H7" t="s">
         <v>11</v>
@@ -651,13 +663,13 @@
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D8">
-        <v>3.4796999999999998</v>
+        <v>1.9616</v>
       </c>
       <c r="E8">
-        <v>229.89</v>
+        <v>229.37</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -677,13 +689,13 @@
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D9">
-        <v>3.0905</v>
+        <v>11.824199999999999</v>
       </c>
       <c r="E9">
-        <v>226.5</v>
+        <v>230.6</v>
       </c>
       <c r="F9">
         <v>1</v>
@@ -697,25 +709,25 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B10" t="s">
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D10">
-        <v>0.62749999999999995</v>
+        <v>3.4796999999999998</v>
       </c>
       <c r="E10">
-        <v>93.27</v>
+        <v>229.89</v>
       </c>
       <c r="F10">
-        <v>4.2350000000000003</v>
+        <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
@@ -723,25 +735,25 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D11">
-        <v>17.255400000000002</v>
+        <v>3.0905</v>
       </c>
       <c r="E11">
-        <v>94.22</v>
+        <v>226.5</v>
       </c>
       <c r="F11">
-        <v>4.2343999999999999</v>
+        <v>1</v>
       </c>
       <c r="G11" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
@@ -755,21 +767,125 @@
         <v>9</v>
       </c>
       <c r="C12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12">
+        <v>0.62749999999999995</v>
+      </c>
+      <c r="E12">
+        <v>93.27</v>
+      </c>
+      <c r="F12">
+        <v>4.2350000000000003</v>
+      </c>
+      <c r="G12" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13">
+        <v>17.255400000000002</v>
+      </c>
+      <c r="E13">
+        <v>94.22</v>
+      </c>
+      <c r="F13">
+        <v>4.2343999999999999</v>
+      </c>
+      <c r="G13" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
         <v>16</v>
       </c>
-      <c r="D12">
+      <c r="D14">
         <v>17.876000000000001</v>
       </c>
-      <c r="E12">
+      <c r="E14">
         <v>94.3</v>
       </c>
-      <c r="F12">
+      <c r="F14">
         <v>4.2874999999999996</v>
       </c>
-      <c r="G12" t="s">
-        <v>10</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="G14" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15">
+        <v>4.6383999999999999</v>
+      </c>
+      <c r="E15">
+        <v>101.3</v>
+      </c>
+      <c r="F15">
+        <v>4.2602000000000002</v>
+      </c>
+      <c r="G15" t="s">
+        <v>10</v>
+      </c>
+      <c r="H15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16">
+        <v>6.7718999999999996</v>
+      </c>
+      <c r="E16">
+        <v>103.78</v>
+      </c>
+      <c r="F16">
+        <v>4.2686000000000002</v>
+      </c>
+      <c r="G16" t="s">
+        <v>10</v>
+      </c>
+      <c r="H16" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>